<commit_message>
Clarify ERP production calculation in TZ
</commit_message>
<xml_diff>
--- a/exports/AERO_TRADE_660-1_fresh_reference_export.xlsx
+++ b/exports/AERO_TRADE_660-1_fresh_reference_export.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Выгрузка" sheetId="1" r:id="R324a40033faf418e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Правила" sheetId="2" r:id="R46d38d605559467a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Выгрузка" sheetId="1" r:id="R02523cfd9b9e4b14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Правила" sheetId="2" r:id="Rc80a790cd5b54866"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1257,7 +1257,7 @@
         <x:v>SUM(Сумма оплаты по строкам блока) - Возмещаемые расходы - Невозмещаемые расходы.</x:v>
       </x:c>
       <x:c r="D9" s="10" t="str">
-        <x:v>Значение считается, а не копируется слепо из Google. Доп. отчеты должны входить в расходы.</x:v>
+        <x:v>Значение считается по ERP-логике. Доп. отчеты должны входить в расходы.</x:v>
       </x:c>
       <x:c r="E9" s="10" t="str">
         <x:v>После учета доп. отчетов delta_check_diff=0 для всех 8 блоков.</x:v>

</xml_diff>